<commit_message>
Improve incubation beast model fit
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -32885,15 +32885,15 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>DragonkinRed1AdamMillerbloodsong</t>
+          <t>DragonChrRedWyrmlingStorvik</t>
         </is>
       </c>
       <c r="J3">
-        <v>1032</v>
+        <v>1668</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Dragonkin: Red 1* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon Chr: Red: Wyrmling* (Storvik)</t>
         </is>
       </c>
       <c r="L3">
@@ -32912,24 +32912,22 @@
           <t>Archhound</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P3">
+        <v>0.48</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact red winged dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact red winged dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -33195,21 +33193,21 @@
         </is>
       </c>
       <c r="P6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Replaced antelope visual with Spineback: Tundra* (PLUSH HYENA of DOOM) during visual review; uses CatDir soundset for a heavier frost-beast profile.</t>
+          <t>Rendered and bounds-checked scale correction; retains Spineback: Tundra* (PLUSH HYENA of DOOM) for the exact tundra Spineback identity at a usable companion scale.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the tundra Spineback silhouette; parent DNA gates incubation only.</t>
+          <t>the exact tundra Spineback identity at a usable companion scale.</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -33381,21 +33379,21 @@
         </is>
       </c>
       <c r="P8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Replaced parrot visual with Spineback: Armour* (PLUSH HYENA of DOOM) during visual review; uses CatDir soundset for a heavier beast profile.</t>
+          <t>Rendered and bounds-checked scale correction; retains Spineback: Armour* (PLUSH HYENA of DOOM) for the exact armoured Spineback identity at a usable companion scale.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the armoured Spineback silhouette; parent DNA gates incubation only.</t>
+          <t>the exact armoured Spineback identity at a usable companion scale.</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -33445,15 +33443,15 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>SpiderDire</t>
+          <t>SpiderDireMediumStorvik</t>
         </is>
       </c>
       <c r="J9">
-        <v>158</v>
+        <v>1902</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Spider: Dire</t>
+          <t>Spider: Dire - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L9">
@@ -33472,24 +33470,22 @@
           <t>SpiderPha</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P9">
+        <v>1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact dark dire-spider silhouette.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact dark dire-spider silhouette.</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -33539,15 +33535,15 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>DragonChrBlack</t>
+          <t>DragonChrBlackWyrmling</t>
         </is>
       </c>
       <c r="J10">
-        <v>41</v>
+        <v>378</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Dragon Chr: Black</t>
+          <t>Dragon Chr: Black: Wyrmling</t>
         </is>
       </c>
       <c r="L10">
@@ -33566,24 +33562,22 @@
           <t>DragonOld</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P10">
+        <v>1</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched black dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched black dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -33754,24 +33748,22 @@
           <t>Werecat</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P12">
+        <v>0.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Cat: Crag Cat for the crag-cat identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the crag-cat identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -33915,15 +33907,15 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>TreantWildWoodsTheAmethystDragon</t>
+          <t>TopiaryGuardianBearTheAmethystDragon</t>
         </is>
       </c>
       <c r="J14">
-        <v>6417</v>
+        <v>6468</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Treant: Wild Woods* (The Amethyst Dragon)</t>
+          <t>Topiary Guardian: Bear* (The Amethyst Dragon)</t>
         </is>
       </c>
       <c r="L14">
@@ -33943,21 +33935,21 @@
         </is>
       </c>
       <c r="P14">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Replaces humanoid fey with a full creature plant silhouette.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a broad bruiser-shaped plant beast rather than a building-sized treant.</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Replaces humanoid fey with a full creature plant silhouette.</t>
+          <t>a broad bruiser-shaped plant beast rather than a building-sized treant.</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -34035,21 +34027,21 @@
         </is>
       </c>
       <c r="P15">
-        <v>1.0</v>
+        <v>0.66</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage Mykal creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Mykal for the canonical SWLOR Mykal silhouette with a manageable wingspan.</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the Mykal appearance and balanced role; parent DNA gates incubation only.</t>
+          <t>the canonical SWLOR Mykal silhouette with a manageable wingspan.</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -34099,15 +34091,15 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Werewolf01</t>
+          <t>DogShadowMastiff</t>
         </is>
       </c>
       <c r="J16">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Werewolf 01</t>
+          <t>Dog: Shadow Mastiff</t>
         </is>
       </c>
       <c r="L16">
@@ -34126,24 +34118,22 @@
           <t>Werewolf</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P16">
+        <v>1</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a dark quadruped prowler instead of a humanoid werewolf.</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a dark quadruped prowler instead of a humanoid werewolf.</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -34193,15 +34183,15 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DragonMetBrass</t>
+          <t>DragonMetBrassWyrmling</t>
         </is>
       </c>
       <c r="J17">
-        <v>42</v>
+        <v>381</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Dragon Met: Brass</t>
+          <t>Dragon Met: Brass: Wyrmling</t>
         </is>
       </c>
       <c r="L17">
@@ -34220,24 +34210,22 @@
           <t>Yuanti</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P17">
+        <v>1</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched brass dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched brass dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -34287,15 +34275,15 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DragonMetCopper</t>
+          <t>DragonMetCopperWyrmling</t>
         </is>
       </c>
       <c r="J18">
-        <v>43</v>
+        <v>382</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Dragon Met: Copper</t>
+          <t>Dragon Met: Copper: Wyrmling</t>
         </is>
       </c>
       <c r="L18">
@@ -34314,24 +34302,22 @@
           <t>LizardM</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P18">
+        <v>1</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched copper dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched copper dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -34381,15 +34367,15 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DragonMetSilver</t>
+          <t>DragonMetSilverWyrmling</t>
         </is>
       </c>
       <c r="J19">
-        <v>44</v>
+        <v>384</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Dragon Met: Silver</t>
+          <t>Dragon Met: Silver: Wyrmling</t>
         </is>
       </c>
       <c r="L19">
@@ -34408,24 +34394,22 @@
           <t>Faerie_Dragon</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P19">
+        <v>1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched silver dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched silver dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -34569,15 +34553,15 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>FeyNymph</t>
+          <t>TopiaryGuardianDeerTheAmethystDragon</t>
         </is>
       </c>
       <c r="J21">
-        <v>126</v>
+        <v>6470</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Fey: Nymph</t>
+          <t>Topiary Guardian: Deer* (The Amethyst Dragon)</t>
         </is>
       </c>
       <c r="L21">
@@ -34596,24 +34580,22 @@
           <t>Archlant</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
+      <c r="P21">
+        <v>1</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; an elegant thorn-covered forest beast instead of a humanoid nymph.</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>an elegant thorn-covered forest beast instead of a humanoid nymph.</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -34690,24 +34672,22 @@
           <t>Horse</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P22">
+        <v>0.85</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Bear: Dire for the dire-bear tank silhouette at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the dire-bear tank silhouette at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -34972,24 +34952,22 @@
           <t>Badger</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P25">
+        <v>0.8</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Myconid: Elder* (Schazzwozzer) for the elder fungal identity at a readable companion height.</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the elder fungal identity at a readable companion height.</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -35006,7 +34984,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Goldmane Sahrak</t>
+          <t>Goldpelt Sahrak</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -35066,24 +35044,22 @@
           <t>House_cat</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P26">
+        <v>0.8</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Golden lioness silhouette retained at 2.98m maximum model extent; no male-lion appearance is installed.</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>Goldpelt describes the available golden lioness exactly and avoids promising a mane the model does not have.</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -35319,15 +35295,15 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SpiderGiant</t>
+          <t>SpiderPhaseLargeStorvik</t>
         </is>
       </c>
       <c r="J29">
-        <v>159</v>
+        <v>1909</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Spider: Giant</t>
+          <t>Spider: Phase - Large* (Storvik)</t>
         </is>
       </c>
       <c r="L29">
@@ -35346,24 +35322,22 @@
           <t>BugbrChf</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P29">
+        <v>1</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a legible large spider that stays inside the companion footprint.</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a legible large spider that stays inside the companion footprint.</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -35413,15 +35387,15 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DragonMetBronze</t>
+          <t>DragonMetBronzeWyrmling</t>
         </is>
       </c>
       <c r="J30">
-        <v>45</v>
+        <v>383</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Dragon Met: Bronze</t>
+          <t>Dragon Met: Bronze: Wyrmling</t>
         </is>
       </c>
       <c r="L30">
@@ -35440,24 +35414,22 @@
           <t>Wolf</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>0.66</t>
-        </is>
+      <c r="P30">
+        <v>1</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched bronze dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched bronze dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -35601,15 +35573,15 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>DragonMetGold</t>
+          <t>DragonMetGoldWyrmling</t>
         </is>
       </c>
       <c r="J32">
-        <v>46</v>
+        <v>385</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Dragon Met: Gold</t>
+          <t>Dragon Met: Gold: Wyrmling</t>
         </is>
       </c>
       <c r="L32">
@@ -35628,24 +35600,22 @@
           <t>Dragon_Prismatic</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P32">
+        <v>1</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched gold dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched gold dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -35883,15 +35853,15 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>DragonChrBlue</t>
+          <t>DragonChrBlueWyrmling</t>
         </is>
       </c>
       <c r="J35">
-        <v>47</v>
+        <v>377</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Dragon Chr: Blue</t>
+          <t>Dragon Chr: Blue: Wyrmling</t>
         </is>
       </c>
       <c r="L35">
@@ -35910,24 +35880,22 @@
           <t>Dragon_Shadow</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
+      <c r="P35">
+        <v>1</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched blue dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched blue dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -36004,24 +35972,22 @@
           <t>Celestial</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P36">
+        <v>0.8</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Cat: Jaguar for the jaguar identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the jaguar identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -36071,15 +36037,15 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Treant1DLATeam</t>
+          <t>ShamblingMound2Hardpoints</t>
         </is>
       </c>
       <c r="J37">
-        <v>1492</v>
+        <v>3893</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Treant 1* (DLA Team)</t>
+          <t>Shambling Mound 2* (Hardpoints)</t>
         </is>
       </c>
       <c r="L37">
@@ -36098,24 +36064,22 @@
           <t>Chicken</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P37">
+        <v>0.65</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Compact, bulky plant silhouette with rooted limbs; scaled to 2.79m maximum model extent.</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>A shambling mound is a literal root-bound colossus while retaining compact creature-space metadata.</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -36165,15 +36129,15 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Wererat</t>
+          <t>RodentRatSewerNitocrisFinniksa</t>
         </is>
       </c>
       <c r="J38">
-        <v>170</v>
+        <v>1983</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Wererat</t>
+          <t>Rodent: Rat: Sewer* (Nitocris&amp;Finniksa)</t>
         </is>
       </c>
       <c r="L38">
@@ -36192,24 +36156,22 @@
           <t>Cow</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P38">
+        <v>1</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a true quadruped sewer-rat silhouette instead of a humanoid lycanthrope.</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a true quadruped sewer-rat silhouette instead of a humanoid lycanthrope.</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
@@ -36756,24 +36718,22 @@
           <t>DoomKngt</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
+      <c r="P44">
+        <v>0.4</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat (NWN) for the distinctive Harat identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the distinctive Harat identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -36823,15 +36783,15 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>BirdEagleIceChild</t>
+          <t>BirdGooseCCP</t>
         </is>
       </c>
       <c r="J45">
-        <v>1275</v>
+        <v>3159</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Bird: Eagle* (Ice-Child)</t>
+          <t>Bird: Goose* (CCP)</t>
         </is>
       </c>
       <c r="L45">
@@ -36851,21 +36811,21 @@
         </is>
       </c>
       <c r="P45">
-        <v>1.0</v>
+        <v>2</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Replaces tiny walking seagull with a stronger flying bird model.</t>
+          <t>Grounded white waterbird silhouette; scaled to 1.43m maximum model extent.</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Replaces tiny walking seagull with a stronger flying bird model.</t>
+          <t>The coastal waterbird form supports both the tide and terrestrial strider elements of the name.</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
@@ -36942,24 +36902,22 @@
           <t>ElemFire</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P46">
+        <v>0.8</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat: Small (NWN) for the small Harat identity without an unexpectedly tall footprint.</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the small Harat identity without an unexpectedly tall footprint.</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -37101,15 +37059,15 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>SpiderPhase</t>
+          <t>SpiderPhaseMediumStorvik</t>
         </is>
       </c>
       <c r="J48">
-        <v>160</v>
+        <v>1908</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Spider: Phase</t>
+          <t>Spider: Phase - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L48">
@@ -37128,24 +37086,22 @@
           <t>Gargoyle</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P48">
+        <v>1</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact phase-spider silhouette.</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact phase-spider silhouette.</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -37287,15 +37243,15 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>SpiderSword</t>
+          <t>SpiderSwordMediumStorvik</t>
         </is>
       </c>
       <c r="J50">
-        <v>161</v>
+        <v>1914</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Spider: Sword</t>
+          <t>Spider: Sword - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L50">
@@ -37314,24 +37270,22 @@
           <t>Ghoullord</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P50">
+        <v>1</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact blade-legged spider silhouette.</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact blade-legged spider silhouette.</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -37381,15 +37335,15 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>DragonkinRed2AdamMillerbloodsong</t>
+          <t>DragonPseudo</t>
         </is>
       </c>
       <c r="J51">
-        <v>1033</v>
+        <v>375</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Dragonkin: Red 2* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon: Pseudo</t>
         </is>
       </c>
       <c r="L51">
@@ -37408,24 +37362,22 @@
           <t>GiantNob</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P51">
+        <v>1</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact reddish flying drake instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact reddish flying drake instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -37475,15 +37427,15 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>DragonkinGreen1AdamMillerbloodsong</t>
+          <t>DragonChrGreenWyrmlingStorvik</t>
         </is>
       </c>
       <c r="J52">
-        <v>1034</v>
+        <v>1656</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Dragonkin: Green 1* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon Chr: Green: Wyrmling* (Storvik)</t>
         </is>
       </c>
       <c r="L52">
@@ -37502,24 +37454,22 @@
           <t>Goblin</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P52">
+        <v>0.8</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact green plated dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact green plated dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -37569,15 +37519,15 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>SpiderWraith</t>
+          <t>SpiderWraithMediumStorvik</t>
         </is>
       </c>
       <c r="J53">
-        <v>162</v>
+        <v>1920</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Spider: Wraith</t>
+          <t>Spider: Wraith - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L53">
@@ -37596,24 +37546,22 @@
           <t>GoblinChf</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P53">
+        <v>1</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact spectral spider silhouette.</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact spectral spider silhouette.</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -37785,21 +37733,21 @@
         </is>
       </c>
       <c r="P55">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Replaces horse model with the requested SWLOR Drex Beast silhouette.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Drex Beast for the canonical SWLOR Drex identity at a readable companion height.</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Replaces horse model with the requested SWLOR Drex Beast silhouette.</t>
+          <t>the canonical SWLOR Drex identity at a readable companion height.</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -37943,15 +37891,15 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>DragonChrGreen</t>
+          <t>DragonChrGreenWyrmling</t>
         </is>
       </c>
       <c r="J57">
-        <v>48</v>
+        <v>379</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Dragon Chr: Green</t>
+          <t>Dragon Chr: Green: Wyrmling</t>
         </is>
       </c>
       <c r="L57">
@@ -37970,24 +37918,22 @@
           <t>GolemIron</t>
         </is>
       </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
+      <c r="P57">
+        <v>1</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched green dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched green dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
@@ -38037,15 +37983,15 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>DragonkinGreen2AdamMillerbloodsong</t>
+          <t>DragonFaerie</t>
         </is>
       </c>
       <c r="J58">
-        <v>1035</v>
+        <v>374</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Dragonkin: Green 2* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon: Faerie</t>
         </is>
       </c>
       <c r="L58">
@@ -38064,24 +38010,22 @@
           <t>GolemStn</t>
         </is>
       </c>
-      <c r="P58" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P58">
+        <v>1</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a small emerald-toned flying dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a small emerald-toned flying dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
@@ -38131,15 +38075,15 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>DragonkinBlue1AdamMillerbloodsong</t>
+          <t>FelldrakeHornedHardpoints</t>
         </is>
       </c>
       <c r="J59">
-        <v>1036</v>
+        <v>3849</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Dragonkin: Blue 1* (Adam Miller &amp; bloodsong)</t>
+          <t>Felldrake: Horned* (Hardpoints)</t>
         </is>
       </c>
       <c r="L59">
@@ -38158,24 +38102,22 @@
           <t>GreyRendr</t>
         </is>
       </c>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P59">
+        <v>0.6</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Dark cobalt-toned quadruped with prominent horns; scaled to 2.89m maximum model extent.</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>The horned felldrake preserves the cobalt palette while making the beast's defining horns unmistakable.</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -38225,15 +38167,15 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>JackalGuardianSzule</t>
+          <t>ZhackalCCCPLUSHHYENAofDOOM</t>
         </is>
       </c>
       <c r="J60">
-        <v>1555</v>
+        <v>3096</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Jackal Guardian* (Szule)</t>
+          <t>Zhackal* (CCC-PLUSH HYENA of DOOM)</t>
         </is>
       </c>
       <c r="L60">
@@ -38253,21 +38195,21 @@
         </is>
       </c>
       <c r="P60">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Replaces generic dog with a distinct predator model.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a lean quadruped jackal predator instead of a humanoid guardian.</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>Replaces generic dog with a distinct predator model.</t>
+          <t>a lean quadruped jackal predator instead of a humanoid guardian.</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
@@ -38409,15 +38351,15 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>DragonkinBlue2AdamMillerbloodsong</t>
+          <t>DragonChrBlueWyrmlingStorvik</t>
         </is>
       </c>
       <c r="J62">
-        <v>1037</v>
+        <v>1596</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Dragonkin: Blue 2* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon Chr: Blue: Wyrmling* (Storvik)</t>
         </is>
       </c>
       <c r="L62">
@@ -38436,24 +38378,22 @@
           <t>Lich</t>
         </is>
       </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="P62">
+        <v>0.7</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Deep sapphire-blue draconic silhouette; scaled to 2.82m maximum model extent.</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>The blue hide makes Sapphireback visually literal without exceeding the gameplay size target.</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
@@ -38595,15 +38535,15 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>DragonChrRed</t>
+          <t>DragonChrRedWyrmling</t>
         </is>
       </c>
       <c r="J64">
-        <v>49</v>
+        <v>376</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Dragon Chr: Red</t>
+          <t>Dragon Chr: Red: Wyrmling</t>
         </is>
       </c>
       <c r="L64">
@@ -38622,24 +38562,22 @@
           <t>LizFemWiz</t>
         </is>
       </c>
-      <c r="P64" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="P64">
+        <v>1</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched red dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched red dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
@@ -38717,21 +38655,21 @@
         </is>
       </c>
       <c r="P65">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Replaced hammerhead shark visual with [SWLOR] Bantha during visual review; uses existing buffalo portrait for better beast-facing UI fit.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Bantha for the canonical SWLOR Bantha identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the Bantha silhouette; parent DNA gates incubation only.</t>
+          <t>the canonical SWLOR Bantha identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">

</xml_diff>

<commit_message>
Synchronize beast lookup visuals
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -36795,11 +36795,11 @@
         </is>
       </c>
       <c r="L45">
-        <v>2224</v>
+        <v>730</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>eagle_</t>
+          <t>seagull_</t>
         </is>
       </c>
       <c r="N45">
@@ -36820,7 +36820,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Grounded white waterbird silhouette; scaled to 1.43m maximum model extent.</t>
+          <t>Grounded white waterbird silhouette; scaled to 1.43m maximum model extent with a matching seagull waterbird portrait.</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">

</xml_diff>

<commit_message>
Match beast portraits and sounds
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -32897,19 +32897,19 @@
         </is>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>632</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>dw_f_01_</t>
+          <t>wyrmlred_</t>
         </is>
       </c>
       <c r="N3">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Archhound</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P3">
@@ -32922,7 +32922,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a compact red winged dragon instead of a humanoid dragonkin.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact red winged dragon instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -33177,11 +33177,11 @@
         </is>
       </c>
       <c r="L6">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>BearBrwn_</t>
+          <t>diretiger_</t>
         </is>
       </c>
       <c r="N6">
@@ -33202,7 +33202,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains Spineback: Tundra* (PLUSH HYENA of DOOM) for the exact tundra Spineback identity at a usable companion scale.</t>
+          <t>Rendered and bounds-checked scale correction; retains Spineback: Tundra* (PLUSH HYENA of DOOM) for the exact tundra Spineback identity at a usable companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -33363,11 +33363,11 @@
         </is>
       </c>
       <c r="L8">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>BearBrwn_</t>
+          <t>diretiger_</t>
         </is>
       </c>
       <c r="N8">
@@ -33388,7 +33388,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains Spineback: Armour* (PLUSH HYENA of DOOM) for the exact armoured Spineback identity at a usable companion scale.</t>
+          <t>Rendered and bounds-checked scale correction; retains Spineback: Armour* (PLUSH HYENA of DOOM) for the exact armoured Spineback identity at a usable companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -33455,19 +33455,19 @@
         </is>
       </c>
       <c r="L9">
-        <v>2094</v>
+        <v>300</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>bugs_</t>
+          <t>SpidDire_</t>
         </is>
       </c>
       <c r="N9">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>SpiderPha</t>
+          <t>SpiderDir</t>
         </is>
       </c>
       <c r="P9">
@@ -33480,7 +33480,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a compact dark dire-spider silhouette.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact dark dire-spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -33547,19 +33547,19 @@
         </is>
       </c>
       <c r="L10">
-        <v>348</v>
+        <v>634</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>yuan_ti_</t>
+          <t>wyrmlblk_</t>
         </is>
       </c>
       <c r="N10">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>DragonOld</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P10">
@@ -33572,7 +33572,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched black dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched black dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -33733,19 +33733,19 @@
         </is>
       </c>
       <c r="L12">
-        <v>314</v>
+        <v>165</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Werecat_</t>
+          <t>cat_crag_</t>
         </is>
       </c>
       <c r="N12">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Werecat</t>
+          <t>CatDir</t>
         </is>
       </c>
       <c r="P12">
@@ -33758,7 +33758,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains Cat: Crag Cat for the crag-cat identity at a large-animal companion scale.</t>
+          <t>Rendered and bounds-checked scale correction; retains Cat: Crag Cat for the crag-cat identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -33919,19 +33919,19 @@
         </is>
       </c>
       <c r="L14">
-        <v>2030</v>
+        <v>181</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>treant_</t>
+          <t>BearDire_</t>
         </is>
       </c>
       <c r="N14">
-        <v>853</v>
+        <v>8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Treant</t>
+          <t>BearDir</t>
         </is>
       </c>
       <c r="P14">
@@ -33944,7 +33944,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a broad bruiser-shaped plant beast rather than a building-sized treant.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a broad bruiser-shaped plant beast rather than a building-sized treant. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -34011,19 +34011,19 @@
         </is>
       </c>
       <c r="L15">
-        <v>184</v>
+        <v>2224</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>DireWolf_</t>
+          <t>eagle_</t>
         </is>
       </c>
       <c r="N15">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Archlant</t>
+          <t>Falcon</t>
         </is>
       </c>
       <c r="P15">
@@ -34036,7 +34036,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Mykal for the canonical SWLOR Mykal silhouette with a manageable wingspan.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Mykal for the canonical SWLOR Mykal silhouette with a manageable wingspan. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -34103,19 +34103,19 @@
         </is>
       </c>
       <c r="L16">
-        <v>151</v>
+        <v>286</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>BlinkDog_</t>
+          <t>ShMastif_</t>
         </is>
       </c>
       <c r="N16">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Werewolf</t>
+          <t>Dog</t>
         </is>
       </c>
       <c r="P16">
@@ -34128,7 +34128,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a dark quadruped prowler instead of a humanoid werewolf.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a dark quadruped prowler instead of a humanoid werewolf. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -34195,19 +34195,19 @@
         </is>
       </c>
       <c r="L17">
-        <v>349</v>
+        <v>637</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Yuanchief_</t>
+          <t>wyrmlbrs_</t>
         </is>
       </c>
       <c r="N17">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Yuanti</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P17">
@@ -34220,7 +34220,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched brass dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched brass dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -34287,19 +34287,19 @@
         </is>
       </c>
       <c r="L18">
-        <v>350</v>
+        <v>638</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Yuanwiz_</t>
+          <t>wyrmlcop_</t>
         </is>
       </c>
       <c r="N18">
-        <v>209</v>
+        <v>30</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>LizardM</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P18">
@@ -34312,7 +34312,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched copper dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched copper dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -34379,19 +34379,19 @@
         </is>
       </c>
       <c r="L19">
-        <v>3499</v>
+        <v>640</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>gldhdragon_</t>
+          <t>wyrmlsil_</t>
         </is>
       </c>
       <c r="N19">
-        <v>330</v>
+        <v>30</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Faerie_Dragon</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P19">
@@ -34404,7 +34404,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched silver dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched silver dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -34565,19 +34565,19 @@
         </is>
       </c>
       <c r="L21">
-        <v>2</v>
+        <v>174</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>dw_f_02_</t>
+          <t>Deer_</t>
         </is>
       </c>
       <c r="N21">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Archlant</t>
+          <t>Deer</t>
         </is>
       </c>
       <c r="P21">
@@ -34590,7 +34590,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; an elegant thorn-covered forest beast instead of a humanoid nymph.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; an elegant thorn-covered forest beast instead of a humanoid nymph. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -34657,19 +34657,19 @@
         </is>
       </c>
       <c r="L22">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>BugbearA_</t>
+          <t>BearDire_</t>
         </is>
       </c>
       <c r="N22">
-        <v>856</v>
+        <v>8</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>BearDir</t>
         </is>
       </c>
       <c r="P22">
@@ -34682,7 +34682,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains Bear: Dire for the dire-bear tank silhouette at a large-animal companion scale.</t>
+          <t>Rendered and bounds-checked scale correction; retains Bear: Dire for the dire-bear tank silhouette at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -34937,19 +34937,19 @@
         </is>
       </c>
       <c r="L25">
-        <v>4</v>
+        <v>2045</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>dw_f_04_</t>
+          <t>Myconid_</t>
         </is>
       </c>
       <c r="N25">
-        <v>4</v>
+        <v>853</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Badger</t>
+          <t>Treant</t>
         </is>
       </c>
       <c r="P25">
@@ -34962,7 +34962,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains Myconid: Elder* (Schazzwozzer) for the elder fungal identity at a readable companion height.</t>
+          <t>Rendered and bounds-checked scale correction; retains Myconid: Elder* (Schazzwozzer) for the elder fungal identity at a readable companion height. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -35029,19 +35029,19 @@
         </is>
       </c>
       <c r="L26">
-        <v>560</v>
+        <v>167</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>BlkPanther_</t>
+          <t>lion_</t>
         </is>
       </c>
       <c r="N26">
-        <v>854</v>
+        <v>18</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>House_cat</t>
+          <t>CatLion</t>
         </is>
       </c>
       <c r="P26">
@@ -35054,7 +35054,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Golden lioness silhouette retained at 2.98m maximum model extent; no male-lion appearance is installed.</t>
+          <t>Golden lioness silhouette retained at 2.98m maximum model extent; no male-lion appearance is installed. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -35307,19 +35307,19 @@
         </is>
       </c>
       <c r="L29">
-        <v>2220</v>
+        <v>302</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>icespider_</t>
+          <t>SpidPhase_</t>
         </is>
       </c>
       <c r="N29">
-        <v>13</v>
+        <v>87</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>BugbrChf</t>
+          <t>SpiderPha</t>
         </is>
       </c>
       <c r="P29">
@@ -35332,7 +35332,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a legible large spider that stays inside the companion footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a legible large spider that stays inside the companion footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -35399,19 +35399,19 @@
         </is>
       </c>
       <c r="L30">
-        <v>316</v>
+        <v>639</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Werewolf_</t>
+          <t>wyrmlbrz_</t>
         </is>
       </c>
       <c r="N30">
-        <v>103</v>
+        <v>30</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Wolf</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P30">
@@ -35424,7 +35424,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched bronze dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched bronze dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -35585,19 +35585,19 @@
         </is>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>641</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>dw_f_05_</t>
+          <t>wyrmlgld_</t>
         </is>
       </c>
       <c r="N32">
-        <v>393</v>
+        <v>30</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Dragon_Prismatic</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P32">
@@ -35610,7 +35610,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched gold dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched gold dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -35865,19 +35865,19 @@
         </is>
       </c>
       <c r="L35">
-        <v>6</v>
+        <v>633</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>dw_f_06_</t>
+          <t>wyrmlblu_</t>
         </is>
       </c>
       <c r="N35">
-        <v>441</v>
+        <v>30</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Dragon_Shadow</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P35">
@@ -35890,7 +35890,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched blue dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched blue dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -35957,19 +35957,19 @@
         </is>
       </c>
       <c r="L36">
-        <v>2154</v>
+        <v>555</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>tiger_</t>
+          <t>cat_jag_</t>
         </is>
       </c>
       <c r="N36">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Celestial</t>
+          <t>CatPanth</t>
         </is>
       </c>
       <c r="P36">
@@ -35982,7 +35982,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains Cat: Jaguar for the jaguar identity at a large-animal companion scale.</t>
+          <t>Rendered and bounds-checked scale correction; retains Cat: Jaguar for the jaguar identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -36049,19 +36049,19 @@
         </is>
       </c>
       <c r="L37">
-        <v>7</v>
+        <v>2035</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>dw_f_07_</t>
+          <t>TwigBlight_</t>
         </is>
       </c>
       <c r="N37">
-        <v>21</v>
+        <v>853</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Chicken</t>
+          <t>Treant</t>
         </is>
       </c>
       <c r="P37">
@@ -36074,7 +36074,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Compact, bulky plant silhouette with rooted limbs; scaled to 2.79m maximum model extent.</t>
+          <t>Compact, bulky plant silhouette with rooted limbs; scaled to 2.79m maximum model extent. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -36149,11 +36149,11 @@
         </is>
       </c>
       <c r="N38">
-        <v>22</v>
+        <v>249</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Cow</t>
+          <t>Rat</t>
         </is>
       </c>
       <c r="P38">
@@ -36166,7 +36166,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a true quadruped sewer-rat silhouette instead of a humanoid lycanthrope.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a true quadruped sewer-rat silhouette instead of a humanoid lycanthrope. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -36703,19 +36703,19 @@
         </is>
       </c>
       <c r="L44">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>horse1a_</t>
+          <t>harat_</t>
         </is>
       </c>
       <c r="N44">
-        <v>28</v>
+        <v>259</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>DoomKngt</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="P44">
@@ -36728,7 +36728,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat (NWN) for the distinctive Harat identity at a large-animal companion scale.</t>
+          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat (NWN) for the distinctive Harat identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -36803,11 +36803,11 @@
         </is>
       </c>
       <c r="N45">
-        <v>38</v>
+        <v>451</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Falcon</t>
+          <t>Seagull</t>
         </is>
       </c>
       <c r="P45">
@@ -36820,7 +36820,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Grounded white waterbird silhouette; scaled to 1.43m maximum model extent with a matching seagull waterbird portrait.</t>
+          <t>Grounded white waterbird silhouette; scaled to 1.43m maximum model extent with a matching seagull waterbird portrait. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -36887,19 +36887,19 @@
         </is>
       </c>
       <c r="L46">
-        <v>1279</v>
+        <v>1276</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>horse1c_</t>
+          <t>harat_</t>
         </is>
       </c>
       <c r="N46">
-        <v>34</v>
+        <v>259</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>ElemFire</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="P46">
@@ -36912,7 +36912,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat: Small (NWN) for the small Harat identity without an unexpectedly tall footprint.</t>
+          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat: Small (NWN) for the small Harat identity without an unexpectedly tall footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -37071,19 +37071,19 @@
         </is>
       </c>
       <c r="L48">
-        <v>10</v>
+        <v>302</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>dw_m_02_</t>
+          <t>SpidPhase_</t>
         </is>
       </c>
       <c r="N48">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Gargoyle</t>
+          <t>SpiderPha</t>
         </is>
       </c>
       <c r="P48">
@@ -37096,7 +37096,7 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a compact phase-spider silhouette.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact phase-spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -37255,19 +37255,19 @@
         </is>
       </c>
       <c r="L50">
-        <v>12</v>
+        <v>303</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>dw_m_04_</t>
+          <t>SpidSwrd_</t>
         </is>
       </c>
       <c r="N50">
-        <v>41</v>
+        <v>88</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Ghoullord</t>
+          <t>SpiderSwd</t>
         </is>
       </c>
       <c r="P50">
@@ -37280,7 +37280,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a compact blade-legged spider silhouette.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact blade-legged spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
@@ -37347,19 +37347,19 @@
         </is>
       </c>
       <c r="L51">
-        <v>13</v>
+        <v>631</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>dw_m_05_</t>
+          <t>drgpseud_</t>
         </is>
       </c>
       <c r="N51">
-        <v>43</v>
+        <v>331</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>GiantNob</t>
+          <t>Pseudodragon</t>
         </is>
       </c>
       <c r="P51">
@@ -37372,7 +37372,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a compact reddish flying drake instead of a humanoid dragonkin.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact reddish flying drake instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -37439,19 +37439,19 @@
         </is>
       </c>
       <c r="L52">
-        <v>14</v>
+        <v>635</v>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>dw_m_06_</t>
+          <t>wyrmlgrn_</t>
         </is>
       </c>
       <c r="N52">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Goblin</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P52">
@@ -37464,7 +37464,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a compact green plated dragon instead of a humanoid dragonkin.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact green plated dragon instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -37531,19 +37531,19 @@
         </is>
       </c>
       <c r="L53">
-        <v>15</v>
+        <v>304</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>dw_m_07_</t>
+          <t>SpidWra_</t>
         </is>
       </c>
       <c r="N53">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>GoblinChf</t>
+          <t>SpiderWra</t>
         </is>
       </c>
       <c r="P53">
@@ -37556,7 +37556,7 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a compact spectral spider silhouette.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact spectral spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -37717,19 +37717,19 @@
         </is>
       </c>
       <c r="L55">
-        <v>356</v>
+        <v>2161</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Zo_War01_</t>
+          <t>drgfiend_</t>
         </is>
       </c>
       <c r="N55">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Curst</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P55">
@@ -37742,7 +37742,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Drex Beast for the canonical SWLOR Drex identity at a readable companion height.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Drex Beast for the canonical SWLOR Drex identity at a readable companion height. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -37903,19 +37903,19 @@
         </is>
       </c>
       <c r="L57">
-        <v>320</v>
+        <v>635</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>WolfWint_</t>
+          <t>wyrmlgrn_</t>
         </is>
       </c>
       <c r="N57">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>GolemIron</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P57">
@@ -37928,7 +37928,7 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched green dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched green dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -37995,19 +37995,19 @@
         </is>
       </c>
       <c r="L58">
-        <v>16</v>
+        <v>630</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>dw_m_08_</t>
+          <t>drgfaerie_</t>
         </is>
       </c>
       <c r="N58">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>GolemStn</t>
+          <t>Faerie_Dragon</t>
         </is>
       </c>
       <c r="P58">
@@ -38020,7 +38020,7 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a small emerald-toned flying dragon instead of a humanoid dragonkin.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a small emerald-toned flying dragon instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -38087,19 +38087,19 @@
         </is>
       </c>
       <c r="L59">
-        <v>17</v>
+        <v>192</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>dw_m_09_</t>
+          <t>DrgBlue_</t>
         </is>
       </c>
       <c r="N59">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>GreyRendr</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P59">
@@ -38112,7 +38112,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Dark cobalt-toned quadruped with prominent horns; scaled to 2.89m maximum model extent.</t>
+          <t>Dark cobalt-toned quadruped with prominent horns; scaled to 2.89m maximum model extent. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -38204,7 +38204,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a lean quadruped jackal predator instead of a humanoid guardian.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a lean quadruped jackal predator instead of a humanoid guardian. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -38363,19 +38363,19 @@
         </is>
       </c>
       <c r="L62">
-        <v>18</v>
+        <v>633</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>el_f_01_</t>
+          <t>wyrmlblu_</t>
         </is>
       </c>
       <c r="N62">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Lich</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P62">
@@ -38388,7 +38388,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Deep sapphire-blue draconic silhouette; scaled to 2.82m maximum model extent.</t>
+          <t>Deep sapphire-blue draconic silhouette; scaled to 2.82m maximum model extent. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -38547,19 +38547,19 @@
         </is>
       </c>
       <c r="L64">
-        <v>2097</v>
+        <v>632</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Owlbear_</t>
+          <t>wyrmlred_</t>
         </is>
       </c>
       <c r="N64">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>LizFemWiz</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P64">
@@ -38572,7 +38572,7 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched red dragon silhouette without an adult dragon footprint.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched red dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
@@ -38664,7 +38664,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Bantha for the canonical SWLOR Bantha identity at a large-animal companion scale.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Bantha for the canonical SWLOR Bantha identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">

</xml_diff>

<commit_message>
Align Goldpelt Sahrak enum identity
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -18867,7 +18867,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>GoldmaneSahrak</t>
+          <t>GoldpeltSahrak</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -34989,7 +34989,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GoldmaneSahrak</t>
+          <t>GoldpeltSahrak</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">

</xml_diff>

<commit_message>
Improve incubation beast model fit (#2210)
* Improve incubation beast model fit

* Complete Goldpelt Sahrak identity rename

* Update Haks companion head

* Synchronize beast lookup visuals

* Match beast portraits and sounds

* Migrate Goldpelt beast names

* Align Goldpelt Sahrak enum identity

* Rebase Goldpelt Haks companion
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -18862,12 +18862,12 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Goldmane Sahrak</t>
+          <t>Goldpelt Sahrak</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>GoldmaneSahrak</t>
+          <t>GoldpeltSahrak</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -32885,51 +32885,49 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>DragonkinRed1AdamMillerbloodsong</t>
+          <t>DragonChrRedWyrmlingStorvik</t>
         </is>
       </c>
       <c r="J3">
-        <v>1032</v>
+        <v>1668</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Dragonkin: Red 1* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon Chr: Red: Wyrmling* (Storvik)</t>
         </is>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>632</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>dw_f_01_</t>
+          <t>wyrmlred_</t>
         </is>
       </c>
       <c r="N3">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Archhound</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P3">
+        <v>0.48</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact red winged dragon instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact red winged dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -33179,11 +33177,11 @@
         </is>
       </c>
       <c r="L6">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>BearBrwn_</t>
+          <t>diretiger_</t>
         </is>
       </c>
       <c r="N6">
@@ -33195,21 +33193,21 @@
         </is>
       </c>
       <c r="P6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Replaced antelope visual with Spineback: Tundra* (PLUSH HYENA of DOOM) during visual review; uses CatDir soundset for a heavier frost-beast profile.</t>
+          <t>Rendered and bounds-checked scale correction; retains Spineback: Tundra* (PLUSH HYENA of DOOM) for the exact tundra Spineback identity at a usable companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the tundra Spineback silhouette; parent DNA gates incubation only.</t>
+          <t>the exact tundra Spineback identity at a usable companion scale.</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -33365,11 +33363,11 @@
         </is>
       </c>
       <c r="L8">
-        <v>148</v>
+        <v>166</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>BearBrwn_</t>
+          <t>diretiger_</t>
         </is>
       </c>
       <c r="N8">
@@ -33381,21 +33379,21 @@
         </is>
       </c>
       <c r="P8">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Replaced parrot visual with Spineback: Armour* (PLUSH HYENA of DOOM) during visual review; uses CatDir soundset for a heavier beast profile.</t>
+          <t>Rendered and bounds-checked scale correction; retains Spineback: Armour* (PLUSH HYENA of DOOM) for the exact armoured Spineback identity at a usable companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the armoured Spineback silhouette; parent DNA gates incubation only.</t>
+          <t>the exact armoured Spineback identity at a usable companion scale.</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -33445,51 +33443,49 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>SpiderDire</t>
+          <t>SpiderDireMediumStorvik</t>
         </is>
       </c>
       <c r="J9">
-        <v>158</v>
+        <v>1902</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Spider: Dire</t>
+          <t>Spider: Dire - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L9">
-        <v>2094</v>
+        <v>300</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>bugs_</t>
+          <t>SpidDire_</t>
         </is>
       </c>
       <c r="N9">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>SpiderPha</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>SpiderDir</t>
+        </is>
+      </c>
+      <c r="P9">
+        <v>1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact dark dire-spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact dark dire-spider silhouette.</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -33539,51 +33535,49 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>DragonChrBlack</t>
+          <t>DragonChrBlackWyrmling</t>
         </is>
       </c>
       <c r="J10">
-        <v>41</v>
+        <v>378</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Dragon Chr: Black</t>
+          <t>Dragon Chr: Black: Wyrmling</t>
         </is>
       </c>
       <c r="L10">
-        <v>348</v>
+        <v>634</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>yuan_ti_</t>
+          <t>wyrmlblk_</t>
         </is>
       </c>
       <c r="N10">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>DragonOld</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P10">
+        <v>1</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched black dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched black dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -33739,39 +33733,37 @@
         </is>
       </c>
       <c r="L12">
-        <v>314</v>
+        <v>165</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Werecat_</t>
+          <t>cat_crag_</t>
         </is>
       </c>
       <c r="N12">
-        <v>98</v>
+        <v>16</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Werecat</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>CatDir</t>
+        </is>
+      </c>
+      <c r="P12">
+        <v>0.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Cat: Crag Cat for the crag-cat identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the crag-cat identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -33915,49 +33907,49 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>TreantWildWoodsTheAmethystDragon</t>
+          <t>TopiaryGuardianBearTheAmethystDragon</t>
         </is>
       </c>
       <c r="J14">
-        <v>6417</v>
+        <v>6468</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Treant: Wild Woods* (The Amethyst Dragon)</t>
+          <t>Topiary Guardian: Bear* (The Amethyst Dragon)</t>
         </is>
       </c>
       <c r="L14">
-        <v>2030</v>
+        <v>181</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>treant_</t>
+          <t>BearDire_</t>
         </is>
       </c>
       <c r="N14">
-        <v>853</v>
+        <v>8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Treant</t>
+          <t>BearDir</t>
         </is>
       </c>
       <c r="P14">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Replaces humanoid fey with a full creature plant silhouette.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a broad bruiser-shaped plant beast rather than a building-sized treant. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Replaces humanoid fey with a full creature plant silhouette.</t>
+          <t>a broad bruiser-shaped plant beast rather than a building-sized treant.</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -34019,37 +34011,37 @@
         </is>
       </c>
       <c r="L15">
-        <v>184</v>
+        <v>2224</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>DireWolf_</t>
+          <t>eagle_</t>
         </is>
       </c>
       <c r="N15">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Archlant</t>
+          <t>Falcon</t>
         </is>
       </c>
       <c r="P15">
-        <v>1.0</v>
+        <v>0.66</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage Mykal creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Mykal for the canonical SWLOR Mykal silhouette with a manageable wingspan. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the Mykal appearance and balanced role; parent DNA gates incubation only.</t>
+          <t>the canonical SWLOR Mykal silhouette with a manageable wingspan.</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -34099,51 +34091,49 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Werewolf01</t>
+          <t>DogShadowMastiff</t>
         </is>
       </c>
       <c r="J16">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Werewolf 01</t>
+          <t>Dog: Shadow Mastiff</t>
         </is>
       </c>
       <c r="L16">
-        <v>151</v>
+        <v>286</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>BlinkDog_</t>
+          <t>ShMastif_</t>
         </is>
       </c>
       <c r="N16">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Werewolf</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Dog</t>
+        </is>
+      </c>
+      <c r="P16">
+        <v>1</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a dark quadruped prowler instead of a humanoid werewolf. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a dark quadruped prowler instead of a humanoid werewolf.</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -34193,51 +34183,49 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DragonMetBrass</t>
+          <t>DragonMetBrassWyrmling</t>
         </is>
       </c>
       <c r="J17">
-        <v>42</v>
+        <v>381</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Dragon Met: Brass</t>
+          <t>Dragon Met: Brass: Wyrmling</t>
         </is>
       </c>
       <c r="L17">
-        <v>349</v>
+        <v>637</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Yuanchief_</t>
+          <t>wyrmlbrs_</t>
         </is>
       </c>
       <c r="N17">
-        <v>108</v>
+        <v>30</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Yuanti</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P17">
+        <v>1</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched brass dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched brass dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -34287,51 +34275,49 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DragonMetCopper</t>
+          <t>DragonMetCopperWyrmling</t>
         </is>
       </c>
       <c r="J18">
-        <v>43</v>
+        <v>382</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Dragon Met: Copper</t>
+          <t>Dragon Met: Copper: Wyrmling</t>
         </is>
       </c>
       <c r="L18">
-        <v>350</v>
+        <v>638</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Yuanwiz_</t>
+          <t>wyrmlcop_</t>
         </is>
       </c>
       <c r="N18">
-        <v>209</v>
+        <v>30</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>LizardM</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P18">
+        <v>1</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched copper dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched copper dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
@@ -34381,51 +34367,49 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DragonMetSilver</t>
+          <t>DragonMetSilverWyrmling</t>
         </is>
       </c>
       <c r="J19">
-        <v>44</v>
+        <v>384</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Dragon Met: Silver</t>
+          <t>Dragon Met: Silver: Wyrmling</t>
         </is>
       </c>
       <c r="L19">
-        <v>3499</v>
+        <v>640</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>gldhdragon_</t>
+          <t>wyrmlsil_</t>
         </is>
       </c>
       <c r="N19">
-        <v>330</v>
+        <v>30</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Faerie_Dragon</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P19">
+        <v>1</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched silver dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched silver dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
@@ -34569,51 +34553,49 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>FeyNymph</t>
+          <t>TopiaryGuardianDeerTheAmethystDragon</t>
         </is>
       </c>
       <c r="J21">
-        <v>126</v>
+        <v>6470</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Fey: Nymph</t>
+          <t>Topiary Guardian: Deer* (The Amethyst Dragon)</t>
         </is>
       </c>
       <c r="L21">
-        <v>2</v>
+        <v>174</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>dw_f_02_</t>
+          <t>Deer_</t>
         </is>
       </c>
       <c r="N21">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Archlant</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
+          <t>Deer</t>
+        </is>
+      </c>
+      <c r="P21">
+        <v>1</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; an elegant thorn-covered forest beast instead of a humanoid nymph. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>an elegant thorn-covered forest beast instead of a humanoid nymph.</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -34675,39 +34657,37 @@
         </is>
       </c>
       <c r="L22">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>BugbearA_</t>
+          <t>BearDire_</t>
         </is>
       </c>
       <c r="N22">
-        <v>856</v>
+        <v>8</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Horse</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>BearDir</t>
+        </is>
+      </c>
+      <c r="P22">
+        <v>0.85</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Bear: Dire for the dire-bear tank silhouette at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the dire-bear tank silhouette at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -34957,39 +34937,37 @@
         </is>
       </c>
       <c r="L25">
-        <v>4</v>
+        <v>2045</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>dw_f_04_</t>
+          <t>Myconid_</t>
         </is>
       </c>
       <c r="N25">
-        <v>4</v>
+        <v>853</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Badger</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Treant</t>
+        </is>
+      </c>
+      <c r="P25">
+        <v>0.8</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Myconid: Elder* (Schazzwozzer) for the elder fungal identity at a readable companion height. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the elder fungal identity at a readable companion height.</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -35006,12 +34984,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Goldmane Sahrak</t>
+          <t>Goldpelt Sahrak</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GoldmaneSahrak</t>
+          <t>GoldpeltSahrak</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -35051,39 +35029,37 @@
         </is>
       </c>
       <c r="L26">
-        <v>560</v>
+        <v>167</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>BlkPanther_</t>
+          <t>lion_</t>
         </is>
       </c>
       <c r="N26">
-        <v>854</v>
+        <v>18</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>House_cat</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>CatLion</t>
+        </is>
+      </c>
+      <c r="P26">
+        <v>0.8</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Golden lioness silhouette retained at 2.98m maximum model extent; no male-lion appearance is installed. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>Goldpelt describes the available golden lioness exactly and avoids promising a mane the model does not have.</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -35319,51 +35295,49 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SpiderGiant</t>
+          <t>SpiderPhaseLargeStorvik</t>
         </is>
       </c>
       <c r="J29">
-        <v>159</v>
+        <v>1909</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Spider: Giant</t>
+          <t>Spider: Phase - Large* (Storvik)</t>
         </is>
       </c>
       <c r="L29">
-        <v>2220</v>
+        <v>302</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>icespider_</t>
+          <t>SpidPhase_</t>
         </is>
       </c>
       <c r="N29">
-        <v>13</v>
+        <v>87</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>BugbrChf</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>SpiderPha</t>
+        </is>
+      </c>
+      <c r="P29">
+        <v>1</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a legible large spider that stays inside the companion footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a legible large spider that stays inside the companion footprint.</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -35413,51 +35387,49 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>DragonMetBronze</t>
+          <t>DragonMetBronzeWyrmling</t>
         </is>
       </c>
       <c r="J30">
-        <v>45</v>
+        <v>383</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Dragon Met: Bronze</t>
+          <t>Dragon Met: Bronze: Wyrmling</t>
         </is>
       </c>
       <c r="L30">
-        <v>316</v>
+        <v>639</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Werewolf_</t>
+          <t>wyrmlbrz_</t>
         </is>
       </c>
       <c r="N30">
-        <v>103</v>
+        <v>30</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Wolf</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>0.66</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P30">
+        <v>1</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched bronze dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched bronze dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -35601,51 +35573,49 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>DragonMetGold</t>
+          <t>DragonMetGoldWyrmling</t>
         </is>
       </c>
       <c r="J32">
-        <v>46</v>
+        <v>385</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Dragon Met: Gold</t>
+          <t>Dragon Met: Gold: Wyrmling</t>
         </is>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>641</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>dw_f_05_</t>
+          <t>wyrmlgld_</t>
         </is>
       </c>
       <c r="N32">
-        <v>393</v>
+        <v>30</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Dragon_Prismatic</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P32">
+        <v>1</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched gold dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched gold dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -35883,51 +35853,49 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>DragonChrBlue</t>
+          <t>DragonChrBlueWyrmling</t>
         </is>
       </c>
       <c r="J35">
-        <v>47</v>
+        <v>377</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Dragon Chr: Blue</t>
+          <t>Dragon Chr: Blue: Wyrmling</t>
         </is>
       </c>
       <c r="L35">
-        <v>6</v>
+        <v>633</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>dw_f_06_</t>
+          <t>wyrmlblu_</t>
         </is>
       </c>
       <c r="N35">
-        <v>441</v>
+        <v>30</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Dragon_Shadow</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P35">
+        <v>1</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched blue dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched blue dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -35989,39 +35957,37 @@
         </is>
       </c>
       <c r="L36">
-        <v>2154</v>
+        <v>555</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>tiger_</t>
+          <t>cat_jag_</t>
         </is>
       </c>
       <c r="N36">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Celestial</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>CatPanth</t>
+        </is>
+      </c>
+      <c r="P36">
+        <v>0.8</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains Cat: Jaguar for the jaguar identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the jaguar identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -36071,51 +36037,49 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Treant1DLATeam</t>
+          <t>ShamblingMound2Hardpoints</t>
         </is>
       </c>
       <c r="J37">
-        <v>1492</v>
+        <v>3893</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Treant 1* (DLA Team)</t>
+          <t>Shambling Mound 2* (Hardpoints)</t>
         </is>
       </c>
       <c r="L37">
-        <v>7</v>
+        <v>2035</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>dw_f_07_</t>
+          <t>TwigBlight_</t>
         </is>
       </c>
       <c r="N37">
-        <v>21</v>
+        <v>853</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Chicken</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Treant</t>
+        </is>
+      </c>
+      <c r="P37">
+        <v>0.65</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Compact, bulky plant silhouette with rooted limbs; scaled to 2.79m maximum model extent. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>A shambling mound is a literal root-bound colossus while retaining compact creature-space metadata.</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -36165,15 +36129,15 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Wererat</t>
+          <t>RodentRatSewerNitocrisFinniksa</t>
         </is>
       </c>
       <c r="J38">
-        <v>170</v>
+        <v>1983</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Wererat</t>
+          <t>Rodent: Rat: Sewer* (Nitocris&amp;Finniksa)</t>
         </is>
       </c>
       <c r="L38">
@@ -36185,31 +36149,29 @@
         </is>
       </c>
       <c r="N38">
-        <v>22</v>
+        <v>249</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Cow</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Rat</t>
+        </is>
+      </c>
+      <c r="P38">
+        <v>1</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a true quadruped sewer-rat silhouette instead of a humanoid lycanthrope. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a true quadruped sewer-rat silhouette instead of a humanoid lycanthrope.</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
@@ -36741,39 +36703,37 @@
         </is>
       </c>
       <c r="L44">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>horse1a_</t>
+          <t>harat_</t>
         </is>
       </c>
       <c r="N44">
-        <v>28</v>
+        <v>259</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>DoomKngt</t>
-        </is>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="P44">
+        <v>0.4</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat (NWN) for the distinctive Harat identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the distinctive Harat identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -36823,49 +36783,49 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>BirdEagleIceChild</t>
+          <t>BirdGooseCCP</t>
         </is>
       </c>
       <c r="J45">
-        <v>1275</v>
+        <v>3159</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Bird: Eagle* (Ice-Child)</t>
+          <t>Bird: Goose* (CCP)</t>
         </is>
       </c>
       <c r="L45">
-        <v>2224</v>
+        <v>730</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>eagle_</t>
+          <t>seagull_</t>
         </is>
       </c>
       <c r="N45">
-        <v>38</v>
+        <v>451</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>Falcon</t>
+          <t>Seagull</t>
         </is>
       </c>
       <c r="P45">
-        <v>1.0</v>
+        <v>2</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Replaces tiny walking seagull with a stronger flying bird model.</t>
+          <t>Grounded white waterbird silhouette; scaled to 1.43m maximum model extent with a matching seagull waterbird portrait. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Replaces tiny walking seagull with a stronger flying bird model.</t>
+          <t>The coastal waterbird form supports both the tide and terrestrial strider elements of the name.</t>
         </is>
       </c>
       <c r="T45" t="inlineStr">
@@ -36927,39 +36887,37 @@
         </is>
       </c>
       <c r="L46">
-        <v>1279</v>
+        <v>1276</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>horse1c_</t>
+          <t>harat_</t>
         </is>
       </c>
       <c r="N46">
-        <v>34</v>
+        <v>259</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>ElemFire</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Horse</t>
+        </is>
+      </c>
+      <c r="P46">
+        <v>0.8</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat: Small (NWN) for the small Harat identity without an unexpectedly tall footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>the small Harat identity without an unexpectedly tall footprint.</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -37101,51 +37059,49 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>SpiderPhase</t>
+          <t>SpiderPhaseMediumStorvik</t>
         </is>
       </c>
       <c r="J48">
-        <v>160</v>
+        <v>1908</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Spider: Phase</t>
+          <t>Spider: Phase - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L48">
-        <v>10</v>
+        <v>302</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>dw_m_02_</t>
+          <t>SpidPhase_</t>
         </is>
       </c>
       <c r="N48">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Gargoyle</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>SpiderPha</t>
+        </is>
+      </c>
+      <c r="P48">
+        <v>1</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact phase-spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact phase-spider silhouette.</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -37287,51 +37243,49 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>SpiderSword</t>
+          <t>SpiderSwordMediumStorvik</t>
         </is>
       </c>
       <c r="J50">
-        <v>161</v>
+        <v>1914</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Spider: Sword</t>
+          <t>Spider: Sword - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L50">
-        <v>12</v>
+        <v>303</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>dw_m_04_</t>
+          <t>SpidSwrd_</t>
         </is>
       </c>
       <c r="N50">
-        <v>41</v>
+        <v>88</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Ghoullord</t>
-        </is>
-      </c>
-      <c r="P50" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>SpiderSwd</t>
+        </is>
+      </c>
+      <c r="P50">
+        <v>1</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact blade-legged spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact blade-legged spider silhouette.</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -37381,51 +37335,49 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>DragonkinRed2AdamMillerbloodsong</t>
+          <t>DragonPseudo</t>
         </is>
       </c>
       <c r="J51">
-        <v>1033</v>
+        <v>375</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Dragonkin: Red 2* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon: Pseudo</t>
         </is>
       </c>
       <c r="L51">
-        <v>13</v>
+        <v>631</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>dw_m_05_</t>
+          <t>drgpseud_</t>
         </is>
       </c>
       <c r="N51">
-        <v>43</v>
+        <v>331</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>GiantNob</t>
-        </is>
-      </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>Pseudodragon</t>
+        </is>
+      </c>
+      <c r="P51">
+        <v>1</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact reddish flying drake instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact reddish flying drake instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -37475,51 +37427,49 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>DragonkinGreen1AdamMillerbloodsong</t>
+          <t>DragonChrGreenWyrmlingStorvik</t>
         </is>
       </c>
       <c r="J52">
-        <v>1034</v>
+        <v>1656</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Dragonkin: Green 1* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon Chr: Green: Wyrmling* (Storvik)</t>
         </is>
       </c>
       <c r="L52">
-        <v>14</v>
+        <v>635</v>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>dw_m_06_</t>
+          <t>wyrmlgrn_</t>
         </is>
       </c>
       <c r="N52">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>Goblin</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P52">
+        <v>0.8</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact green plated dragon instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact green plated dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -37569,51 +37519,49 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>SpiderWraith</t>
+          <t>SpiderWraithMediumStorvik</t>
         </is>
       </c>
       <c r="J53">
-        <v>162</v>
+        <v>1920</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Spider: Wraith</t>
+          <t>Spider: Wraith - Medium* (Storvik)</t>
         </is>
       </c>
       <c r="L53">
-        <v>15</v>
+        <v>304</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>dw_m_07_</t>
+          <t>SpidWra_</t>
         </is>
       </c>
       <c r="N53">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>GoblinChf</t>
-        </is>
-      </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>SpiderWra</t>
+        </is>
+      </c>
+      <c r="P53">
+        <v>1</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a compact spectral spider silhouette. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a compact spectral spider silhouette.</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -37769,37 +37717,37 @@
         </is>
       </c>
       <c r="L55">
-        <v>356</v>
+        <v>2161</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Zo_War01_</t>
+          <t>drgfiend_</t>
         </is>
       </c>
       <c r="N55">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>Curst</t>
+          <t>DragonYng</t>
         </is>
       </c>
       <c r="P55">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Replaces horse model with the requested SWLOR Drex Beast silhouette.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Drex Beast for the canonical SWLOR Drex identity at a readable companion height. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Replaces horse model with the requested SWLOR Drex Beast silhouette.</t>
+          <t>the canonical SWLOR Drex identity at a readable companion height.</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -37943,51 +37891,49 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>DragonChrGreen</t>
+          <t>DragonChrGreenWyrmling</t>
         </is>
       </c>
       <c r="J57">
-        <v>48</v>
+        <v>379</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Dragon Chr: Green</t>
+          <t>Dragon Chr: Green: Wyrmling</t>
         </is>
       </c>
       <c r="L57">
-        <v>320</v>
+        <v>635</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>WolfWint_</t>
+          <t>wyrmlgrn_</t>
         </is>
       </c>
       <c r="N57">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>GolemIron</t>
-        </is>
-      </c>
-      <c r="P57" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P57">
+        <v>1</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched green dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched green dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T57" t="inlineStr">
@@ -38037,51 +37983,49 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>DragonkinGreen2AdamMillerbloodsong</t>
+          <t>DragonFaerie</t>
         </is>
       </c>
       <c r="J58">
-        <v>1035</v>
+        <v>374</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Dragonkin: Green 2* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon: Faerie</t>
         </is>
       </c>
       <c r="L58">
-        <v>16</v>
+        <v>630</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>dw_m_08_</t>
+          <t>drgfaerie_</t>
         </is>
       </c>
       <c r="N58">
-        <v>50</v>
+        <v>330</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>GolemStn</t>
-        </is>
-      </c>
-      <c r="P58" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>Faerie_Dragon</t>
+        </is>
+      </c>
+      <c r="P58">
+        <v>1</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a small emerald-toned flying dragon instead of a humanoid dragonkin. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a small emerald-toned flying dragon instead of a humanoid dragonkin.</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
@@ -38131,51 +38075,49 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>DragonkinBlue1AdamMillerbloodsong</t>
+          <t>FelldrakeHornedHardpoints</t>
         </is>
       </c>
       <c r="J59">
-        <v>1036</v>
+        <v>3849</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Dragonkin: Blue 1* (Adam Miller &amp; bloodsong)</t>
+          <t>Felldrake: Horned* (Hardpoints)</t>
         </is>
       </c>
       <c r="L59">
-        <v>17</v>
+        <v>192</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>dw_m_09_</t>
+          <t>DrgBlue_</t>
         </is>
       </c>
       <c r="N59">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>GreyRendr</t>
-        </is>
-      </c>
-      <c r="P59" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P59">
+        <v>0.6</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Dark cobalt-toned quadruped with prominent horns; scaled to 2.89m maximum model extent. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>The horned felldrake preserves the cobalt palette while making the beast's defining horns unmistakable.</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
@@ -38225,15 +38167,15 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>JackalGuardianSzule</t>
+          <t>ZhackalCCCPLUSHHYENAofDOOM</t>
         </is>
       </c>
       <c r="J60">
-        <v>1555</v>
+        <v>3096</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Jackal Guardian* (Szule)</t>
+          <t>Zhackal* (CCC-PLUSH HYENA of DOOM)</t>
         </is>
       </c>
       <c r="L60">
@@ -38253,21 +38195,21 @@
         </is>
       </c>
       <c r="P60">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Approved replacement</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Replaces generic dog with a distinct predator model.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a lean quadruped jackal predator instead of a humanoid guardian. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>Replaces generic dog with a distinct predator model.</t>
+          <t>a lean quadruped jackal predator instead of a humanoid guardian.</t>
         </is>
       </c>
       <c r="T60" t="inlineStr">
@@ -38409,51 +38351,49 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>DragonkinBlue2AdamMillerbloodsong</t>
+          <t>DragonChrBlueWyrmlingStorvik</t>
         </is>
       </c>
       <c r="J62">
-        <v>1037</v>
+        <v>1596</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Dragonkin: Blue 2* (Adam Miller &amp; bloodsong)</t>
+          <t>Dragon Chr: Blue: Wyrmling* (Storvik)</t>
         </is>
       </c>
       <c r="L62">
-        <v>18</v>
+        <v>633</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>el_f_01_</t>
+          <t>wyrmlblu_</t>
         </is>
       </c>
       <c r="N62">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>Lich</t>
-        </is>
-      </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P62">
+        <v>0.7</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after name-fit audit</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Deep sapphire-blue draconic silhouette; scaled to 2.82m maximum model extent. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>The blue hide makes Sapphireback visually literal without exceeding the gameplay size target.</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
@@ -38595,51 +38535,49 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>DragonChrRed</t>
+          <t>DragonChrRedWyrmling</t>
         </is>
       </c>
       <c r="J64">
-        <v>49</v>
+        <v>376</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Dragon Chr: Red</t>
+          <t>Dragon Chr: Red: Wyrmling</t>
         </is>
       </c>
       <c r="L64">
-        <v>2097</v>
+        <v>632</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>Owlbear_</t>
+          <t>wyrmlred_</t>
         </is>
       </c>
       <c r="N64">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>LizFemWiz</t>
-        </is>
-      </c>
-      <c r="P64" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>DragonYng</t>
+        </is>
+      </c>
+      <c r="P64">
+        <v>1</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Unused by current beast rows; selected as a standalone second-stage creature asset. Requires in-game visual review before implementation.</t>
+          <t>Rendered and bounds-checked replacement for the previous appearance; a color-matched red dragon silhouette without an adult dragon footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the chosen appearance and role; parent DNA gates incubation only.</t>
+          <t>a color-matched red dragon silhouette without an adult dragon footprint.</t>
         </is>
       </c>
       <c r="T64" t="inlineStr">
@@ -38717,21 +38655,21 @@
         </is>
       </c>
       <c r="P65">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Selected Candidate</t>
+          <t>Approved after visual audit</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Replaced hammerhead shark visual with [SWLOR] Bantha during visual review; uses existing buffalo portrait for better beast-facing UI fit.</t>
+          <t>Rendered and bounds-checked scale correction; retains [SWLOR] Bantha for the canonical SWLOR Bantha identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>Standalone second-stage identity selected for the Bantha silhouette; parent DNA gates incubation only.</t>
+          <t>the canonical SWLOR Bantha identity at a large-animal companion scale.</t>
         </is>
       </c>
       <c r="T65" t="inlineStr">

</xml_diff>

<commit_message>
Fix duplicate incubation beast visuals
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -36691,49 +36691,49 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>UniqueHaratNWN</t>
+          <t>CattleBisonFinniksaNitocris</t>
         </is>
       </c>
       <c r="J44">
-        <v>461</v>
+        <v>1015</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>[Unique] Harat (NWN)</t>
+          <t>Cattle: Bison* (Finniksa&amp;Nitocris)</t>
         </is>
       </c>
       <c r="L44">
-        <v>1276</v>
+        <v>2004</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>harat_</t>
+          <t>bison_</t>
         </is>
       </c>
       <c r="N44">
-        <v>259</v>
+        <v>22</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Cow</t>
         </is>
       </c>
       <c r="P44">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Approved after visual audit</t>
+          <t>Selected after live visual correction</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat (NWN) for the distinctive Harat identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
+          <t>Installed brown bison quadruped selected after the Harat rendered in game as an oversized winged humanoid. The 0.8 scale keeps the large-animal mutation within a normal companion footprint; portrait and sound use installed bison/cattle assets.</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>the distinctive Harat identity at a large-animal companion scale.</t>
+          <t>A brown, heavy quadruped preserves the amber hide and Ronto-derived large-animal identity without a humanoid silhouette.</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -36875,49 +36875,49 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>UniqueHaratSmallNWN</t>
+          <t>Wolverinehydromancerx</t>
         </is>
       </c>
       <c r="J46">
-        <v>462</v>
+        <v>1337</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>[Unique] Harat: Small (NWN)</t>
+          <t>Wolverine* (hydromancerx)</t>
         </is>
       </c>
       <c r="L46">
-        <v>1276</v>
+        <v>2206</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>harat_</t>
+          <t>wolverine_</t>
         </is>
       </c>
       <c r="N46">
-        <v>259</v>
+        <v>5</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>BadgerDir</t>
         </is>
       </c>
       <c r="P46">
-        <v>0.8</v>
+        <v>1.25</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Approved after visual audit</t>
+          <t>Selected after live visual correction</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat: Small (NWN) for the small Harat identity without an unexpectedly tall footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
+          <t>Installed wolverine quadruped selected after the small Harat rendered in game as the same oversized winged humanoid. The 1.25 scale keeps the compact mustelid readable beside a player; portrait and sound use installed wolverine/dire-badger assets.</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>the small Harat identity without an unexpectedly tall footprint.</t>
+          <t>A soot-brown mustelid is a distinct, compact bruiser mutation of Scrap Rat and matches the Mirekit name without reusing a humanoid silhouette.</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -41549,6 +41549,66 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Appearance</t>
+        </is>
+      </c>
+      <c r="B66">
+        <v>461</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>UniqueHaratNWN</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>[Unique] Harat (NWN)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Rejected after live in-game review: the model renders as an oversized winged humanoid and does not read as an animal companion.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Rejected for incubation beasts</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Appearance</t>
+        </is>
+      </c>
+      <c r="B67">
+        <v>462</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>UniqueHaratSmallNWN</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>[Unique] Harat: Small (NWN)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Rejected after live in-game review: this row renders as the same oversized winged humanoid as the full Harat appearance, so it does not provide a distinct small-beast silhouette.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Rejected for incubation beasts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F38"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Extend rejected asset sheet controls
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -41610,9 +41610,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F38"/>
+  <autoFilter ref="A1:F67"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A65">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A67">
       <formula1>"Appearance,Portrait,Soundset"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix duplicate incubation beast visuals (#2212)
* Fix duplicate incubation beast visuals

* Sync beast level visual source data

* Extend rejected asset sheet controls
</commit_message>
<xml_diff>
--- a/design/bible/SWLOR Design Bible - Private Source Data.xlsx
+++ b/design/bible/SWLOR Design Bible - Private Source Data.xlsx
@@ -36691,49 +36691,49 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>UniqueHaratNWN</t>
+          <t>CattleBisonFinniksaNitocris</t>
         </is>
       </c>
       <c r="J44">
-        <v>461</v>
+        <v>1015</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>[Unique] Harat (NWN)</t>
+          <t>Cattle: Bison* (Finniksa&amp;Nitocris)</t>
         </is>
       </c>
       <c r="L44">
-        <v>1276</v>
+        <v>2004</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>harat_</t>
+          <t>bison_</t>
         </is>
       </c>
       <c r="N44">
-        <v>259</v>
+        <v>22</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Cow</t>
         </is>
       </c>
       <c r="P44">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Approved after visual audit</t>
+          <t>Selected after live visual correction</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat (NWN) for the distinctive Harat identity at a large-animal companion scale. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
+          <t>Installed brown bison quadruped selected after the Harat rendered in game as an oversized winged humanoid. The 0.8 scale keeps the large-animal mutation within a normal companion footprint; portrait and sound use installed bison/cattle assets.</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>the distinctive Harat identity at a large-animal companion scale.</t>
+          <t>A brown, heavy quadruped preserves the amber hide and Ronto-derived large-animal identity without a humanoid silhouette.</t>
         </is>
       </c>
       <c r="T44" t="inlineStr">
@@ -36875,49 +36875,49 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>UniqueHaratSmallNWN</t>
+          <t>Wolverinehydromancerx</t>
         </is>
       </c>
       <c r="J46">
-        <v>462</v>
+        <v>1337</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>[Unique] Harat: Small (NWN)</t>
+          <t>Wolverine* (hydromancerx)</t>
         </is>
       </c>
       <c r="L46">
-        <v>1276</v>
+        <v>2206</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>harat_</t>
+          <t>wolverine_</t>
         </is>
       </c>
       <c r="N46">
-        <v>259</v>
+        <v>5</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>BadgerDir</t>
         </is>
       </c>
       <c r="P46">
-        <v>0.8</v>
+        <v>1.25</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Approved after visual audit</t>
+          <t>Selected after live visual correction</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Rendered and bounds-checked scale correction; retains [Unique] Harat: Small (NWN) for the small Harat identity without an unexpectedly tall footprint. Portrait and sound set were audited against installed 2DA creature assets and matched to the selected appearance.</t>
+          <t>Installed wolverine quadruped selected after the small Harat rendered in game as the same oversized winged humanoid. The 1.25 scale keeps the compact mustelid readable beside a player; portrait and sound use installed wolverine/dire-badger assets.</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>the small Harat identity without an unexpectedly tall footprint.</t>
+          <t>A soot-brown mustelid is a distinct, compact bruiser mutation of Scrap Rat and matches the Mirekit name without reusing a humanoid silhouette.</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -41549,10 +41549,70 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Appearance</t>
+        </is>
+      </c>
+      <c r="B66">
+        <v>461</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>UniqueHaratNWN</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>[Unique] Harat (NWN)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Rejected after live in-game review: the model renders as an oversized winged humanoid and does not read as an animal companion.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Rejected for incubation beasts</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Appearance</t>
+        </is>
+      </c>
+      <c r="B67">
+        <v>462</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>UniqueHaratSmallNWN</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>[Unique] Harat: Small (NWN)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Rejected after live in-game review: this row renders as the same oversized winged humanoid as the full Harat appearance, so it does not provide a distinct small-beast silhouette.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Rejected for incubation beasts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F38"/>
+  <autoFilter ref="A1:F67"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A65">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A67">
       <formula1>"Appearance,Portrait,Soundset"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>